<commit_message>
Changed additional file upon contributor email request
</commit_message>
<xml_diff>
--- a/_data/supplementary/2a5bfa3b7fe561a117010ab4_Novus_Biological_Porcine_Adiponectin_ELISA/Porcine_Adiponectin_Novus_Biological_09_24_2026.xlsx
+++ b/_data/supplementary/2a5bfa3b7fe561a117010ab4_Novus_Biological_Porcine_Adiponectin_ELISA/Porcine_Adiponectin_Novus_Biological_09_24_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mstate-my.sharepoint.com/personal/ma2020_msstate_edu/Documents/Documents 1/ELISA Project/Submit to the equine registry/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="93" documentId="11_F972590FBB44245486E6AA5B7054D7BEA2B1F7D5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B186934-26EE-4E31-B894-BE6F435B2941}"/>
+  <xr:revisionPtr revIDLastSave="97" documentId="11_F972590FBB44245486E6AA5B7054D7BEA2B1F7D5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{256DFC27-F11C-4208-9656-F9D054BA9194}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -807,18 +807,6 @@
     <t>Spike 4 (Serum 400X</t>
   </si>
   <si>
-    <t>Spike 1 (EtOH 1X)</t>
-  </si>
-  <si>
-    <t>Spike 2 (EtOH 25X)</t>
-  </si>
-  <si>
-    <t>Spike 3 (EtOH 100X)</t>
-  </si>
-  <si>
-    <t>Spike 4 (EtOH 400X</t>
-  </si>
-  <si>
     <t>Spikes Preparation</t>
   </si>
   <si>
@@ -838,6 +826,18 @@
   </si>
   <si>
     <t>Sp = spike</t>
+  </si>
+  <si>
+    <t>Spike 5 (EtOH 1X)</t>
+  </si>
+  <si>
+    <t>Spike 6 (EtOH 25X)</t>
+  </si>
+  <si>
+    <t>Spike 7 (EtOH 100X)</t>
+  </si>
+  <si>
+    <t>Spike 8 (EtOH 400X</t>
   </si>
 </sst>
 </file>
@@ -1090,10 +1090,10 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2047,13 +2047,13 @@
     </row>
     <row r="31" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F31" s="39" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="G31" s="39"/>
     </row>
     <row r="32" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F32" s="40" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="G32" s="40"/>
     </row>
@@ -2123,7 +2123,7 @@
       </c>
     </row>
     <row r="5" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="44" t="s">
+      <c r="A5" s="43" t="s">
         <v>8</v>
       </c>
       <c r="B5" s="11" t="s">
@@ -2144,15 +2144,15 @@
       <c r="G5" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="H5" s="43"/>
-      <c r="I5" s="43"/>
-      <c r="J5" s="43"/>
-      <c r="K5" s="43"/>
-      <c r="L5" s="43"/>
-      <c r="M5" s="43"/>
+      <c r="H5" s="44"/>
+      <c r="I5" s="44"/>
+      <c r="J5" s="44"/>
+      <c r="K5" s="44"/>
+      <c r="L5" s="44"/>
+      <c r="M5" s="44"/>
     </row>
     <row r="6" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="43"/>
+      <c r="A6" s="44"/>
       <c r="B6" s="13" t="s">
         <v>204</v>
       </c>
@@ -2171,15 +2171,15 @@
       <c r="G6" s="14" t="s">
         <v>204</v>
       </c>
-      <c r="H6" s="43"/>
-      <c r="I6" s="43"/>
-      <c r="J6" s="43"/>
-      <c r="K6" s="43"/>
-      <c r="L6" s="43"/>
-      <c r="M6" s="43"/>
+      <c r="H6" s="44"/>
+      <c r="I6" s="44"/>
+      <c r="J6" s="44"/>
+      <c r="K6" s="44"/>
+      <c r="L6" s="44"/>
+      <c r="M6" s="44"/>
     </row>
     <row r="7" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="43"/>
+      <c r="A7" s="44"/>
       <c r="B7" s="15" t="s">
         <v>205</v>
       </c>
@@ -2198,15 +2198,15 @@
       <c r="G7" s="16" t="s">
         <v>206</v>
       </c>
-      <c r="H7" s="43"/>
-      <c r="I7" s="43"/>
-      <c r="J7" s="43"/>
-      <c r="K7" s="43"/>
-      <c r="L7" s="43"/>
-      <c r="M7" s="43"/>
+      <c r="H7" s="44"/>
+      <c r="I7" s="44"/>
+      <c r="J7" s="44"/>
+      <c r="K7" s="44"/>
+      <c r="L7" s="44"/>
+      <c r="M7" s="44"/>
     </row>
     <row r="8" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="44" t="s">
+      <c r="A8" s="43" t="s">
         <v>9</v>
       </c>
       <c r="B8" s="11" t="s">
@@ -2227,15 +2227,15 @@
       <c r="G8" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="H8" s="43"/>
-      <c r="I8" s="43"/>
-      <c r="J8" s="43"/>
-      <c r="K8" s="43"/>
-      <c r="L8" s="43"/>
-      <c r="M8" s="43"/>
+      <c r="H8" s="44"/>
+      <c r="I8" s="44"/>
+      <c r="J8" s="44"/>
+      <c r="K8" s="44"/>
+      <c r="L8" s="44"/>
+      <c r="M8" s="44"/>
     </row>
     <row r="9" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="43"/>
+      <c r="A9" s="44"/>
       <c r="B9" s="13" t="s">
         <v>204</v>
       </c>
@@ -2254,15 +2254,15 @@
       <c r="G9" s="14" t="s">
         <v>204</v>
       </c>
-      <c r="H9" s="43"/>
-      <c r="I9" s="43"/>
-      <c r="J9" s="43"/>
-      <c r="K9" s="43"/>
-      <c r="L9" s="43"/>
-      <c r="M9" s="43"/>
+      <c r="H9" s="44"/>
+      <c r="I9" s="44"/>
+      <c r="J9" s="44"/>
+      <c r="K9" s="44"/>
+      <c r="L9" s="44"/>
+      <c r="M9" s="44"/>
     </row>
     <row r="10" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="43"/>
+      <c r="A10" s="44"/>
       <c r="B10" s="15" t="s">
         <v>207</v>
       </c>
@@ -2281,15 +2281,15 @@
       <c r="G10" s="16" t="s">
         <v>206</v>
       </c>
-      <c r="H10" s="43"/>
-      <c r="I10" s="43"/>
-      <c r="J10" s="43"/>
-      <c r="K10" s="43"/>
-      <c r="L10" s="43"/>
-      <c r="M10" s="43"/>
+      <c r="H10" s="44"/>
+      <c r="I10" s="44"/>
+      <c r="J10" s="44"/>
+      <c r="K10" s="44"/>
+      <c r="L10" s="44"/>
+      <c r="M10" s="44"/>
     </row>
     <row r="11" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="44" t="s">
+      <c r="A11" s="43" t="s">
         <v>10</v>
       </c>
       <c r="B11" s="11" t="s">
@@ -2310,15 +2310,15 @@
       <c r="G11" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="H11" s="43"/>
-      <c r="I11" s="43"/>
-      <c r="J11" s="43"/>
-      <c r="K11" s="43"/>
-      <c r="L11" s="43"/>
-      <c r="M11" s="43"/>
+      <c r="H11" s="44"/>
+      <c r="I11" s="44"/>
+      <c r="J11" s="44"/>
+      <c r="K11" s="44"/>
+      <c r="L11" s="44"/>
+      <c r="M11" s="44"/>
     </row>
     <row r="12" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="43"/>
+      <c r="A12" s="44"/>
       <c r="B12" s="13" t="s">
         <v>204</v>
       </c>
@@ -2337,15 +2337,15 @@
       <c r="G12" s="14" t="s">
         <v>204</v>
       </c>
-      <c r="H12" s="43"/>
-      <c r="I12" s="43"/>
-      <c r="J12" s="43"/>
-      <c r="K12" s="43"/>
-      <c r="L12" s="43"/>
-      <c r="M12" s="43"/>
+      <c r="H12" s="44"/>
+      <c r="I12" s="44"/>
+      <c r="J12" s="44"/>
+      <c r="K12" s="44"/>
+      <c r="L12" s="44"/>
+      <c r="M12" s="44"/>
     </row>
     <row r="13" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="43"/>
+      <c r="A13" s="44"/>
       <c r="B13" s="15" t="s">
         <v>208</v>
       </c>
@@ -2364,15 +2364,15 @@
       <c r="G13" s="16" t="s">
         <v>206</v>
       </c>
-      <c r="H13" s="43"/>
-      <c r="I13" s="43"/>
-      <c r="J13" s="43"/>
-      <c r="K13" s="43"/>
-      <c r="L13" s="43"/>
-      <c r="M13" s="43"/>
+      <c r="H13" s="44"/>
+      <c r="I13" s="44"/>
+      <c r="J13" s="44"/>
+      <c r="K13" s="44"/>
+      <c r="L13" s="44"/>
+      <c r="M13" s="44"/>
     </row>
     <row r="14" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="44" t="s">
+      <c r="A14" s="43" t="s">
         <v>11</v>
       </c>
       <c r="B14" s="11" t="s">
@@ -2393,15 +2393,15 @@
       <c r="G14" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="H14" s="43"/>
-      <c r="I14" s="43"/>
-      <c r="J14" s="43"/>
-      <c r="K14" s="43"/>
-      <c r="L14" s="43"/>
-      <c r="M14" s="43"/>
+      <c r="H14" s="44"/>
+      <c r="I14" s="44"/>
+      <c r="J14" s="44"/>
+      <c r="K14" s="44"/>
+      <c r="L14" s="44"/>
+      <c r="M14" s="44"/>
     </row>
     <row r="15" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="43"/>
+      <c r="A15" s="44"/>
       <c r="B15" s="13" t="s">
         <v>204</v>
       </c>
@@ -2420,15 +2420,15 @@
       <c r="G15" s="14" t="s">
         <v>204</v>
       </c>
-      <c r="H15" s="43"/>
-      <c r="I15" s="43"/>
-      <c r="J15" s="43"/>
-      <c r="K15" s="43"/>
-      <c r="L15" s="43"/>
-      <c r="M15" s="43"/>
+      <c r="H15" s="44"/>
+      <c r="I15" s="44"/>
+      <c r="J15" s="44"/>
+      <c r="K15" s="44"/>
+      <c r="L15" s="44"/>
+      <c r="M15" s="44"/>
     </row>
     <row r="16" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="43"/>
+      <c r="A16" s="44"/>
       <c r="B16" s="15" t="s">
         <v>209</v>
       </c>
@@ -2447,15 +2447,15 @@
       <c r="G16" s="16" t="s">
         <v>206</v>
       </c>
-      <c r="H16" s="43"/>
-      <c r="I16" s="43"/>
-      <c r="J16" s="43"/>
-      <c r="K16" s="43"/>
-      <c r="L16" s="43"/>
-      <c r="M16" s="43"/>
+      <c r="H16" s="44"/>
+      <c r="I16" s="44"/>
+      <c r="J16" s="44"/>
+      <c r="K16" s="44"/>
+      <c r="L16" s="44"/>
+      <c r="M16" s="44"/>
     </row>
     <row r="17" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="44" t="s">
+      <c r="A17" s="43" t="s">
         <v>12</v>
       </c>
       <c r="B17" s="11" t="s">
@@ -2476,15 +2476,15 @@
       <c r="G17" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="H17" s="43"/>
-      <c r="I17" s="43"/>
-      <c r="J17" s="43"/>
-      <c r="K17" s="43"/>
-      <c r="L17" s="43"/>
-      <c r="M17" s="43"/>
+      <c r="H17" s="44"/>
+      <c r="I17" s="44"/>
+      <c r="J17" s="44"/>
+      <c r="K17" s="44"/>
+      <c r="L17" s="44"/>
+      <c r="M17" s="44"/>
     </row>
     <row r="18" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="43"/>
+      <c r="A18" s="44"/>
       <c r="B18" s="13" t="s">
         <v>204</v>
       </c>
@@ -2503,15 +2503,15 @@
       <c r="G18" s="14" t="s">
         <v>204</v>
       </c>
-      <c r="H18" s="43"/>
-      <c r="I18" s="43"/>
-      <c r="J18" s="43"/>
-      <c r="K18" s="43"/>
-      <c r="L18" s="43"/>
-      <c r="M18" s="43"/>
+      <c r="H18" s="44"/>
+      <c r="I18" s="44"/>
+      <c r="J18" s="44"/>
+      <c r="K18" s="44"/>
+      <c r="L18" s="44"/>
+      <c r="M18" s="44"/>
     </row>
     <row r="19" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="43"/>
+      <c r="A19" s="44"/>
       <c r="B19" s="15" t="s">
         <v>210</v>
       </c>
@@ -2530,15 +2530,15 @@
       <c r="G19" s="16" t="s">
         <v>206</v>
       </c>
-      <c r="H19" s="43"/>
-      <c r="I19" s="43"/>
-      <c r="J19" s="43"/>
-      <c r="K19" s="43"/>
-      <c r="L19" s="43"/>
-      <c r="M19" s="43"/>
+      <c r="H19" s="44"/>
+      <c r="I19" s="44"/>
+      <c r="J19" s="44"/>
+      <c r="K19" s="44"/>
+      <c r="L19" s="44"/>
+      <c r="M19" s="44"/>
     </row>
     <row r="20" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="44" t="s">
+      <c r="A20" s="43" t="s">
         <v>13</v>
       </c>
       <c r="B20" s="11" t="s">
@@ -2559,15 +2559,15 @@
       <c r="G20" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="H20" s="43"/>
-      <c r="I20" s="43"/>
-      <c r="J20" s="43"/>
-      <c r="K20" s="43"/>
-      <c r="L20" s="43"/>
-      <c r="M20" s="43"/>
+      <c r="H20" s="44"/>
+      <c r="I20" s="44"/>
+      <c r="J20" s="44"/>
+      <c r="K20" s="44"/>
+      <c r="L20" s="44"/>
+      <c r="M20" s="44"/>
     </row>
     <row r="21" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="43"/>
+      <c r="A21" s="44"/>
       <c r="B21" s="13" t="s">
         <v>204</v>
       </c>
@@ -2586,15 +2586,15 @@
       <c r="G21" s="14" t="s">
         <v>204</v>
       </c>
-      <c r="H21" s="43"/>
-      <c r="I21" s="43"/>
-      <c r="J21" s="43"/>
-      <c r="K21" s="43"/>
-      <c r="L21" s="43"/>
-      <c r="M21" s="43"/>
+      <c r="H21" s="44"/>
+      <c r="I21" s="44"/>
+      <c r="J21" s="44"/>
+      <c r="K21" s="44"/>
+      <c r="L21" s="44"/>
+      <c r="M21" s="44"/>
     </row>
     <row r="22" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="43"/>
+      <c r="A22" s="44"/>
       <c r="B22" s="15" t="s">
         <v>211</v>
       </c>
@@ -2613,15 +2613,15 @@
       <c r="G22" s="16" t="s">
         <v>206</v>
       </c>
-      <c r="H22" s="43"/>
-      <c r="I22" s="43"/>
-      <c r="J22" s="43"/>
-      <c r="K22" s="43"/>
-      <c r="L22" s="43"/>
-      <c r="M22" s="43"/>
+      <c r="H22" s="44"/>
+      <c r="I22" s="44"/>
+      <c r="J22" s="44"/>
+      <c r="K22" s="44"/>
+      <c r="L22" s="44"/>
+      <c r="M22" s="44"/>
     </row>
     <row r="23" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="44" t="s">
+      <c r="A23" s="43" t="s">
         <v>14</v>
       </c>
       <c r="B23" s="11" t="s">
@@ -2642,15 +2642,15 @@
       <c r="G23" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="H23" s="43"/>
-      <c r="I23" s="43"/>
-      <c r="J23" s="43"/>
-      <c r="K23" s="43"/>
-      <c r="L23" s="43"/>
-      <c r="M23" s="43"/>
+      <c r="H23" s="44"/>
+      <c r="I23" s="44"/>
+      <c r="J23" s="44"/>
+      <c r="K23" s="44"/>
+      <c r="L23" s="44"/>
+      <c r="M23" s="44"/>
     </row>
     <row r="24" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="43"/>
+      <c r="A24" s="44"/>
       <c r="B24" s="13" t="s">
         <v>204</v>
       </c>
@@ -2669,15 +2669,15 @@
       <c r="G24" s="14" t="s">
         <v>204</v>
       </c>
-      <c r="H24" s="43"/>
-      <c r="I24" s="43"/>
-      <c r="J24" s="43"/>
-      <c r="K24" s="43"/>
-      <c r="L24" s="43"/>
-      <c r="M24" s="43"/>
+      <c r="H24" s="44"/>
+      <c r="I24" s="44"/>
+      <c r="J24" s="44"/>
+      <c r="K24" s="44"/>
+      <c r="L24" s="44"/>
+      <c r="M24" s="44"/>
     </row>
     <row r="25" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="43"/>
+      <c r="A25" s="44"/>
       <c r="B25" s="15" t="s">
         <v>212</v>
       </c>
@@ -2696,15 +2696,15 @@
       <c r="G25" s="16" t="s">
         <v>206</v>
       </c>
-      <c r="H25" s="43"/>
-      <c r="I25" s="43"/>
-      <c r="J25" s="43"/>
-      <c r="K25" s="43"/>
-      <c r="L25" s="43"/>
-      <c r="M25" s="43"/>
+      <c r="H25" s="44"/>
+      <c r="I25" s="44"/>
+      <c r="J25" s="44"/>
+      <c r="K25" s="44"/>
+      <c r="L25" s="44"/>
+      <c r="M25" s="44"/>
     </row>
     <row r="26" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="44" t="s">
+      <c r="A26" s="43" t="s">
         <v>15</v>
       </c>
       <c r="B26" s="17" t="s">
@@ -2725,15 +2725,15 @@
       <c r="G26" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="H26" s="43"/>
-      <c r="I26" s="43"/>
-      <c r="J26" s="43"/>
-      <c r="K26" s="43"/>
-      <c r="L26" s="43"/>
-      <c r="M26" s="43"/>
+      <c r="H26" s="44"/>
+      <c r="I26" s="44"/>
+      <c r="J26" s="44"/>
+      <c r="K26" s="44"/>
+      <c r="L26" s="44"/>
+      <c r="M26" s="44"/>
     </row>
     <row r="27" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="43"/>
+      <c r="A27" s="44"/>
       <c r="B27" s="18" t="s">
         <v>204</v>
       </c>
@@ -2752,15 +2752,15 @@
       <c r="G27" s="14" t="s">
         <v>204</v>
       </c>
-      <c r="H27" s="43"/>
-      <c r="I27" s="43"/>
-      <c r="J27" s="43"/>
-      <c r="K27" s="43"/>
-      <c r="L27" s="43"/>
-      <c r="M27" s="43"/>
+      <c r="H27" s="44"/>
+      <c r="I27" s="44"/>
+      <c r="J27" s="44"/>
+      <c r="K27" s="44"/>
+      <c r="L27" s="44"/>
+      <c r="M27" s="44"/>
     </row>
     <row r="28" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="43"/>
+      <c r="A28" s="44"/>
       <c r="B28" s="19"/>
       <c r="C28" s="16" t="s">
         <v>206</v>
@@ -2777,12 +2777,12 @@
       <c r="G28" s="16" t="s">
         <v>206</v>
       </c>
-      <c r="H28" s="43"/>
-      <c r="I28" s="43"/>
-      <c r="J28" s="43"/>
-      <c r="K28" s="43"/>
-      <c r="L28" s="43"/>
-      <c r="M28" s="43"/>
+      <c r="H28" s="44"/>
+      <c r="I28" s="44"/>
+      <c r="J28" s="44"/>
+      <c r="K28" s="44"/>
+      <c r="L28" s="44"/>
+      <c r="M28" s="44"/>
     </row>
     <row r="33" spans="1:1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
@@ -2791,6 +2791,46 @@
     </row>
   </sheetData>
   <mergeCells count="56">
+    <mergeCell ref="M20:M22"/>
+    <mergeCell ref="M23:M25"/>
+    <mergeCell ref="M26:M28"/>
+    <mergeCell ref="M5:M7"/>
+    <mergeCell ref="M8:M10"/>
+    <mergeCell ref="M11:M13"/>
+    <mergeCell ref="M14:M16"/>
+    <mergeCell ref="M17:M19"/>
+    <mergeCell ref="K20:K22"/>
+    <mergeCell ref="K23:K25"/>
+    <mergeCell ref="K26:K28"/>
+    <mergeCell ref="L5:L7"/>
+    <mergeCell ref="L8:L10"/>
+    <mergeCell ref="L11:L13"/>
+    <mergeCell ref="L14:L16"/>
+    <mergeCell ref="L17:L19"/>
+    <mergeCell ref="L20:L22"/>
+    <mergeCell ref="L23:L25"/>
+    <mergeCell ref="L26:L28"/>
+    <mergeCell ref="K5:K7"/>
+    <mergeCell ref="K8:K10"/>
+    <mergeCell ref="K11:K13"/>
+    <mergeCell ref="K14:K16"/>
+    <mergeCell ref="K17:K19"/>
+    <mergeCell ref="I20:I22"/>
+    <mergeCell ref="I23:I25"/>
+    <mergeCell ref="I26:I28"/>
+    <mergeCell ref="J5:J7"/>
+    <mergeCell ref="J8:J10"/>
+    <mergeCell ref="J11:J13"/>
+    <mergeCell ref="J14:J16"/>
+    <mergeCell ref="J17:J19"/>
+    <mergeCell ref="J20:J22"/>
+    <mergeCell ref="J23:J25"/>
+    <mergeCell ref="J26:J28"/>
+    <mergeCell ref="I5:I7"/>
+    <mergeCell ref="I8:I10"/>
+    <mergeCell ref="I11:I13"/>
+    <mergeCell ref="I14:I16"/>
+    <mergeCell ref="I17:I19"/>
     <mergeCell ref="A20:A22"/>
     <mergeCell ref="A23:A25"/>
     <mergeCell ref="A26:A28"/>
@@ -2807,46 +2847,6 @@
     <mergeCell ref="A11:A13"/>
     <mergeCell ref="A14:A16"/>
     <mergeCell ref="A17:A19"/>
-    <mergeCell ref="I20:I22"/>
-    <mergeCell ref="I23:I25"/>
-    <mergeCell ref="I26:I28"/>
-    <mergeCell ref="J5:J7"/>
-    <mergeCell ref="J8:J10"/>
-    <mergeCell ref="J11:J13"/>
-    <mergeCell ref="J14:J16"/>
-    <mergeCell ref="J17:J19"/>
-    <mergeCell ref="J20:J22"/>
-    <mergeCell ref="J23:J25"/>
-    <mergeCell ref="J26:J28"/>
-    <mergeCell ref="I5:I7"/>
-    <mergeCell ref="I8:I10"/>
-    <mergeCell ref="I11:I13"/>
-    <mergeCell ref="I14:I16"/>
-    <mergeCell ref="I17:I19"/>
-    <mergeCell ref="K20:K22"/>
-    <mergeCell ref="K23:K25"/>
-    <mergeCell ref="K26:K28"/>
-    <mergeCell ref="L5:L7"/>
-    <mergeCell ref="L8:L10"/>
-    <mergeCell ref="L11:L13"/>
-    <mergeCell ref="L14:L16"/>
-    <mergeCell ref="L17:L19"/>
-    <mergeCell ref="L20:L22"/>
-    <mergeCell ref="L23:L25"/>
-    <mergeCell ref="L26:L28"/>
-    <mergeCell ref="K5:K7"/>
-    <mergeCell ref="K8:K10"/>
-    <mergeCell ref="K11:K13"/>
-    <mergeCell ref="K14:K16"/>
-    <mergeCell ref="K17:K19"/>
-    <mergeCell ref="M20:M22"/>
-    <mergeCell ref="M23:M25"/>
-    <mergeCell ref="M26:M28"/>
-    <mergeCell ref="M5:M7"/>
-    <mergeCell ref="M8:M10"/>
-    <mergeCell ref="M11:M13"/>
-    <mergeCell ref="M14:M16"/>
-    <mergeCell ref="M17:M19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4129,13 +4129,13 @@
         <v>96</v>
       </c>
       <c r="F103" s="39" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="G103" s="39"/>
     </row>
     <row r="104" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F104" s="40" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="G104" s="40"/>
     </row>
@@ -4636,13 +4636,13 @@
     </row>
     <row r="34" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F34" s="39" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="G34" s="39"/>
     </row>
     <row r="35" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F35" s="40" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="G35" s="40"/>
     </row>
@@ -5693,7 +5693,7 @@
         <v>112.01287499999999</v>
       </c>
       <c r="N86" s="42" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="O86" s="42"/>
       <c r="P86" s="42"/>
@@ -5722,16 +5722,16 @@
         <v>95</v>
       </c>
       <c r="N87" s="37" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="O87" s="37" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="P87" s="37" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="Q87" s="38" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
     </row>
     <row r="88" spans="1:17" ht="12.75" x14ac:dyDescent="0.2">
@@ -6089,7 +6089,7 @@
         <v>236</v>
       </c>
       <c r="I100" s="20" t="s">
-        <v>254</v>
+        <v>261</v>
       </c>
       <c r="J100" s="21">
         <v>40</v>
@@ -6125,7 +6125,7 @@
         <v>240</v>
       </c>
       <c r="I101" s="20" t="s">
-        <v>255</v>
+        <v>262</v>
       </c>
       <c r="J101" s="21">
         <v>40</v>
@@ -6140,7 +6140,7 @@
     </row>
     <row r="102" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="I102" s="20" t="s">
-        <v>256</v>
+        <v>263</v>
       </c>
       <c r="J102" s="21">
         <v>40</v>
@@ -6158,11 +6158,11 @@
         <v>96</v>
       </c>
       <c r="F103" s="39" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="G103" s="39"/>
       <c r="I103" s="20" t="s">
-        <v>257</v>
+        <v>264</v>
       </c>
       <c r="J103" s="21">
         <v>40</v>
@@ -6177,7 +6177,7 @@
     </row>
     <row r="104" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F104" s="40" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="G104" s="40"/>
     </row>

</xml_diff>